<commit_message>
no title all caps
</commit_message>
<xml_diff>
--- a/keydates/2026_election_admin_dates_deadlines.xlsx
+++ b/keydates/2026_election_admin_dates_deadlines.xlsx
@@ -1,14 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brennancenterny-my.sharepoint.com/personal/zhangj_brennan_law_nyu_edu/Documents/Documents/2026_midterms/keydates/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_55A37B9D72D90932D66DE0E1A282A0810564D2F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65DC5C57-CA25-3042-9B6B-7E3CB664DDCA}"/>
+  <bookViews>
+    <workbookView xWindow="45380" yWindow="840" windowWidth="26760" windowHeight="20420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="2026_election_admin_dates_deadl" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Early Voting Data" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Early Voting Daily Totals" sheetId="3" r:id="rId7"/>
+    <sheet name="2026_election_admin_dates_deadl" sheetId="1" r:id="rId1"/>
+    <sheet name="Early Voting Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Early Voting Daily Totals" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -1056,29 +1065,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1086,66 +1109,56 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1335,17 +1348,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:K59"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1380,1657 +1396,1657 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="5">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="C2" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D2" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="E2" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F2" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="G2" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="H2" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I2" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="C3" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="D3" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E3" s="5">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="G3" s="5">
-        <v>46344.0</v>
+        <v>46344</v>
       </c>
       <c r="I3" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="J3" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K3" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B4" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C4" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D4" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F4" s="5">
-        <v>46334.0</v>
+        <v>46334</v>
       </c>
       <c r="G4" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H4" s="5">
-        <v>46345.0</v>
+        <v>46345</v>
       </c>
       <c r="I4" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J4" s="4">
-        <v>46302.0</v>
+        <v>46302</v>
       </c>
       <c r="K4" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="C5" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D5" s="5">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="E5" s="5">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="G5" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="H5" s="5">
-        <v>46344.0</v>
+        <v>46344</v>
       </c>
       <c r="I5" s="5">
-        <v>46374.0</v>
+        <v>46374</v>
       </c>
       <c r="J5" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K5" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B6" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C6" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="D6" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E6" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F6" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="G6" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="H6" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="I6" s="5">
-        <v>46367.0</v>
+        <v>46367</v>
       </c>
       <c r="J6" s="4">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="K6" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B7" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C7" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D7" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F7" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="G7" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="H7" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="I7" s="5">
-        <v>46356.0</v>
+        <v>46356</v>
       </c>
       <c r="J7" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K7" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B8" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C8" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D8" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="E8" s="5">
-        <v>46298.0</v>
+        <v>46298</v>
       </c>
       <c r="G8" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H8" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="I8" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="J8" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K8" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B9" s="5">
-        <v>46305.0</v>
+        <v>46305</v>
       </c>
       <c r="C9" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D9" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E9" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="F9" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G9" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H9" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="I9" s="5">
-        <v>46334.0</v>
+        <v>46334</v>
       </c>
       <c r="J9" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="K9" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C10" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="D10" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F10" s="5">
-        <v>46345.0</v>
+        <v>46345</v>
       </c>
       <c r="G10" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I10" s="5">
-        <v>46358.0</v>
+        <v>46358</v>
       </c>
       <c r="J10" s="4">
-        <v>46317.0</v>
+        <v>46317</v>
       </c>
       <c r="K10" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B11" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C11" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D11" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F11" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="G11" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="H11" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="I11" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="J11" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K11" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B12" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C12" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D12" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E12" s="5">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="F12" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="G12" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="H12" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="I12" s="5">
-        <v>46346.0</v>
+        <v>46346</v>
       </c>
       <c r="J12" s="4">
-        <v>46307.0</v>
+        <v>46307</v>
       </c>
       <c r="K12" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B13" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C13" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D13" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E13" s="5">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="F13" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="G13" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H13" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="I13" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J13" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K13" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B14" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C14" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D14" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G14" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H14" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="I14" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="J14" s="4">
-        <v>46307.0</v>
+        <v>46307</v>
       </c>
       <c r="K14" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B15" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C15" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="D15" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F15" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="G15" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="H15" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="I15" s="5">
-        <v>46360.0</v>
+        <v>46360</v>
       </c>
       <c r="J15" s="4">
-        <v>46289.0</v>
+        <v>46289</v>
       </c>
       <c r="K15" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B16" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C16" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D16" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F16" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="G16" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="H16" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="I16" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="J16" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="K16" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
         <v>96</v>
       </c>
       <c r="B17" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C17" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D17" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E17" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F17" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="G17" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="H17" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="I17" s="5">
-        <v>46356.0</v>
+        <v>46356</v>
       </c>
       <c r="J17" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="K17" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B18" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="C18" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="D18" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G18" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H18" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="I18" s="5">
-        <v>46357.0</v>
+        <v>46357</v>
       </c>
       <c r="J18" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="K18" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B19" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C19" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D19" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E19" s="5">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="F19" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G19" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H19" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="I19" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J19" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="K19" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B20" s="5">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="C20" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="D20" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="E20" s="5">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="G20" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H20" s="5">
-        <v>46334.0</v>
+        <v>46334</v>
       </c>
       <c r="I20" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J20" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K20" s="4">
-        <v>46322.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1" t="s">
         <v>115</v>
       </c>
       <c r="B21" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C21" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D21" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E21" s="5">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="F21" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G21" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H21" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="I21" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J21" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="K21" s="4">
-        <v>46324.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B22" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C22" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="D22" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E22" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="F22" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="G22" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="H22" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I22" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="J22" s="4">
-        <v>46317.0</v>
+        <v>46317</v>
       </c>
       <c r="K22" s="4">
-        <v>46324.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1" t="s">
         <v>126</v>
       </c>
       <c r="B23" s="5">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="C23" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="D23" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E23" s="5">
-        <v>46320.0</v>
+        <v>46320</v>
       </c>
       <c r="G23" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="H23" s="5">
-        <v>46344.0</v>
+        <v>46344</v>
       </c>
       <c r="I23" s="5">
-        <v>46360.0</v>
+        <v>46360</v>
       </c>
       <c r="J23" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="K23" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B24" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C24" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D24" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E24" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F24" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="G24" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="H24" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="I24" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J24" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="K24" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B25" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C25" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D25" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E25" s="5">
-        <v>46310.0</v>
+        <v>46310</v>
       </c>
       <c r="G25" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H25" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="I25" s="5">
-        <v>46345.0</v>
+        <v>46345</v>
       </c>
       <c r="J25" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="K25" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B26" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C26" s="5">
-        <v>46334.0</v>
+        <v>46334</v>
       </c>
       <c r="D26" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E26" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G26" s="5">
-        <v>46334.0</v>
+        <v>46334</v>
       </c>
       <c r="H26" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I26" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="J26" s="4"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B27" s="5">
-        <v>46302.0</v>
+        <v>46302</v>
       </c>
       <c r="C27" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D27" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E27" s="5">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="G27" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="H27" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="I27" s="5">
-        <v>46364.0</v>
+        <v>46364</v>
       </c>
       <c r="J27" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K27" s="3"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B28" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C28" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D28" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E28" s="5">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F28" s="5">
-        <v>46330.0</v>
+        <v>46330</v>
       </c>
       <c r="G28" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H28" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="I28" s="5">
-        <v>46356.0</v>
+        <v>46356</v>
       </c>
       <c r="J28" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="K28" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1" t="s">
         <v>154</v>
       </c>
       <c r="B29" s="5">
-        <v>46318.0</v>
+        <v>46318</v>
       </c>
       <c r="C29" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D29" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E29" s="5">
-        <v>46318.0</v>
+        <v>46318</v>
       </c>
       <c r="G29" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H29" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="I29" s="5">
-        <v>46356.0</v>
+        <v>46356</v>
       </c>
       <c r="J29" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="K29" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B30" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C30" s="5">
-        <v>46333.0</v>
+        <v>46333</v>
       </c>
       <c r="D30" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F30" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="G30" s="5">
-        <v>46333.0</v>
+        <v>46333</v>
       </c>
       <c r="H30" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I30" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="J30" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="K30" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1" t="s">
         <v>164</v>
       </c>
       <c r="B31" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C31" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D31" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E31" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G31" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H31" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="I31" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="1" t="s">
         <v>170</v>
       </c>
       <c r="B32" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="C32" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="D32" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E32" s="5">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F32" s="5">
-        <v>46340.0</v>
+        <v>46340</v>
       </c>
       <c r="G32" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="H32" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="I32" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="J32" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="K32" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="1" t="s">
         <v>176</v>
       </c>
       <c r="B33" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C33" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D33" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E33" s="5">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F33" s="5">
-        <v>46346.0</v>
+        <v>46346</v>
       </c>
       <c r="G33" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H33" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I33" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="J33" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="K33" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="1" t="s">
         <v>181</v>
       </c>
       <c r="B34" s="5">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="C34" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="D34" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E34" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="G34" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="H34" s="5">
-        <v>46354.0</v>
+        <v>46354</v>
       </c>
       <c r="I34" s="5">
-        <v>46371.0</v>
+        <v>46371</v>
       </c>
       <c r="J34" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="K34" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="1" t="s">
         <v>187</v>
       </c>
       <c r="B35" s="5">
-        <v>46304.0</v>
+        <v>46304</v>
       </c>
       <c r="C35" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D35" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E35" s="5">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="F35" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="G35" s="5">
-        <v>46338.0</v>
+        <v>46338</v>
       </c>
       <c r="H35" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I35" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="J35" s="4">
-        <v>46310.0</v>
+        <v>46310</v>
       </c>
       <c r="K35" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="1" t="s">
         <v>192</v>
       </c>
       <c r="C36" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D36" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E36" s="5">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F36" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="G36" s="5">
-        <v>46341.0</v>
+        <v>46341</v>
       </c>
       <c r="H36" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="I36" s="5">
-        <v>46346.0</v>
+        <v>46346</v>
       </c>
       <c r="J36" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="K36" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="1" t="s">
         <v>197</v>
       </c>
       <c r="B37" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="C37" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D37" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F37" s="5">
-        <v>46333.0</v>
+        <v>46333</v>
       </c>
       <c r="G37" s="5">
-        <v>46333.0</v>
+        <v>46333</v>
       </c>
       <c r="H37" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="I37" s="5">
-        <v>46360.0</v>
+        <v>46360</v>
       </c>
       <c r="J37" s="4">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="K37" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="1" t="s">
         <v>201</v>
       </c>
       <c r="B38" s="5">
-        <v>46304.0</v>
+        <v>46304</v>
       </c>
       <c r="C38" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D38" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="E38" s="5">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="G38" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H38" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="I38" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J38" s="4">
-        <v>46323.0</v>
+        <v>46323</v>
       </c>
       <c r="K38" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="1" t="s">
         <v>206</v>
       </c>
       <c r="B39" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="C39" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="D39" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F39" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="G39" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="H39" s="5">
-        <v>46356.0</v>
+        <v>46356</v>
       </c>
       <c r="I39" s="5">
-        <v>46366.0</v>
+        <v>46366</v>
       </c>
       <c r="J39" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="K39" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B40" s="5">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="C40" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D40" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E40" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G40" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="H40" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J40" s="4">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="K40" s="4">
-        <v>46322.0</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="1" t="s">
         <v>216</v>
       </c>
       <c r="B41" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="C41" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D41" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E41" s="5">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="F41" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="G41" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="H41" s="5">
-        <v>46330.0</v>
+        <v>46330</v>
       </c>
       <c r="J41" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="K41" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="1" t="s">
         <v>218</v>
       </c>
       <c r="B42" s="5">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="C42" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D42" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E42" s="5">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="G42" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="H42" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="I42" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="J42" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K42" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="1" t="s">
         <v>222</v>
       </c>
       <c r="B43" s="5">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="C43" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D43" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E43" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="G43" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H43" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="I43" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J43" s="4">
-        <v>46283.0</v>
+        <v>46283</v>
       </c>
       <c r="K43" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B44" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C44" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G44" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H44" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="I44" s="5">
-        <v>46351.0</v>
+        <v>46351</v>
       </c>
       <c r="J44" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="K44" s="4">
-        <v>46324.0</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="1" t="s">
         <v>232</v>
       </c>
       <c r="B45" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="C45" s="5">
-        <v>46330.0</v>
+        <v>46330</v>
       </c>
       <c r="D45" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E45" s="5">
-        <v>46321.0</v>
+        <v>46321</v>
       </c>
       <c r="F45" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="G45" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="H45" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="I45" s="5">
-        <v>46363.0</v>
+        <v>46363</v>
       </c>
       <c r="J45" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="K45" s="4">
-        <v>46325.0</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B46" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C46" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D46" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F46" s="5">
-        <v>46342.0</v>
+        <v>46342</v>
       </c>
       <c r="G46" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H46" s="5">
-        <v>46343.0</v>
+        <v>46343</v>
       </c>
       <c r="I46" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="J46" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K46" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B47" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C47" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D47" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E47" s="5">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="F47" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G47" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H47" s="5">
-        <v>46331.0</v>
+        <v>46331</v>
       </c>
       <c r="I47" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J47" s="4">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="K47" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="1" t="s">
         <v>245</v>
       </c>
       <c r="B48" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C48" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="D48" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F48" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="G48" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="H48" s="5">
-        <v>46339.0</v>
+        <v>46339</v>
       </c>
       <c r="I48" s="5">
-        <v>46363.0</v>
+        <v>46363</v>
       </c>
       <c r="J48" s="4">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="K48" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="1" t="s">
         <v>250</v>
       </c>
       <c r="B49" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C49" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="D49" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F49" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="G49" s="5">
-        <v>46349.0</v>
+        <v>46349</v>
       </c>
       <c r="H49" s="5">
-        <v>46350.0</v>
+        <v>46350</v>
       </c>
       <c r="I49" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="J49" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="K49" s="4">
-        <v>46329.0</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="1" t="s">
         <v>254</v>
       </c>
       <c r="B50" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="C50" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="D50" s="5">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="E50" s="5">
-        <v>46316.0</v>
+        <v>46316</v>
       </c>
       <c r="G50" s="5">
-        <v>46335.0</v>
+        <v>46335</v>
       </c>
       <c r="H50" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="I50" s="5">
-        <v>46359.0</v>
+        <v>46359</v>
       </c>
       <c r="J50" s="4">
-        <v>46316.0</v>
+        <v>46316</v>
       </c>
       <c r="K50" s="4">
-        <v>46326.0</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="1" t="s">
         <v>260</v>
       </c>
       <c r="B51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="G51" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="I51" s="5">
-        <v>46357.0</v>
+        <v>46357</v>
       </c>
       <c r="J51" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="K51" s="4">
-        <v>46327.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>46327</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="1" t="s">
         <v>265</v>
       </c>
       <c r="B52" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="C52" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="D52" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="E52" s="5">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="G52" s="5">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="H52" s="5">
-        <v>46332.0</v>
+        <v>46332</v>
       </c>
       <c r="I52" s="5">
-        <v>46336.0</v>
+        <v>46336</v>
       </c>
       <c r="J52" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="K52" s="4">
-        <v>46328.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="1" t="s">
         <v>273</v>
       </c>
@@ -3038,7 +3054,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="1" t="s">
         <v>309</v>
       </c>
@@ -3046,7 +3062,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="1" t="s">
         <v>335</v>
       </c>
@@ -3066,22 +3082,30 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B57"/>
-    <hyperlink r:id="rId2" ref="B58"/>
-    <hyperlink r:id="rId3" ref="B59"/>
+    <hyperlink ref="B57" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B58" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B59" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
-  <drawing r:id="rId4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" customWidth="1"/>
+    <col min="7" max="7" width="28.1640625" customWidth="1"/>
+    <col min="8" max="8" width="36" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -3110,7 +3134,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -3118,13 +3142,13 @@
         <v>22</v>
       </c>
       <c r="C2" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>24</v>
@@ -3139,7 +3163,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
@@ -3147,13 +3171,13 @@
         <v>29</v>
       </c>
       <c r="C3" s="4">
-        <v>46302.0</v>
+        <v>46302</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>31</v>
@@ -3168,7 +3192,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>34</v>
       </c>
@@ -3176,13 +3200,13 @@
         <v>22</v>
       </c>
       <c r="C4" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E4" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>37</v>
@@ -3197,7 +3221,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
@@ -3205,13 +3229,13 @@
         <v>42</v>
       </c>
       <c r="C5" s="4">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>44</v>
@@ -3226,7 +3250,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
         <v>43</v>
       </c>
@@ -3234,13 +3258,13 @@
         <v>49</v>
       </c>
       <c r="C6" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E6" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>50</v>
@@ -3255,7 +3279,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
@@ -3263,13 +3287,13 @@
         <v>22</v>
       </c>
       <c r="C7" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E7" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>56</v>
@@ -3284,7 +3308,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>53</v>
       </c>
@@ -3292,13 +3316,13 @@
         <v>61</v>
       </c>
       <c r="C8" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>62</v>
       </c>
       <c r="E8" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>63</v>
@@ -3313,7 +3337,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
         <v>57</v>
       </c>
@@ -3321,13 +3345,13 @@
         <v>68</v>
       </c>
       <c r="C9" s="4">
-        <v>46317.0</v>
+        <v>46317</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E9" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>71</v>
@@ -3342,7 +3366,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
         <v>64</v>
       </c>
@@ -3350,13 +3374,13 @@
         <v>76</v>
       </c>
       <c r="C10" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>77</v>
       </c>
       <c r="E10" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>78</v>
@@ -3371,7 +3395,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
         <v>69</v>
       </c>
@@ -3379,13 +3403,13 @@
         <v>83</v>
       </c>
       <c r="C11" s="4">
-        <v>46307.0</v>
+        <v>46307</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>85</v>
       </c>
       <c r="E11" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>86</v>
@@ -3400,7 +3424,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
         <v>75</v>
       </c>
@@ -3408,13 +3432,13 @@
         <v>91</v>
       </c>
       <c r="C12" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>92</v>
       </c>
       <c r="E12" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>93</v>
@@ -3429,7 +3453,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
         <v>80</v>
       </c>
@@ -3437,13 +3461,13 @@
         <v>98</v>
       </c>
       <c r="C13" s="4">
-        <v>46307.0</v>
+        <v>46307</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>99</v>
       </c>
       <c r="E13" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>100</v>
@@ -3458,7 +3482,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
         <v>84</v>
       </c>
@@ -3466,13 +3490,13 @@
         <v>104</v>
       </c>
       <c r="C14" s="4">
-        <v>46289.0</v>
+        <v>46289</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>106</v>
       </c>
       <c r="E14" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>107</v>
@@ -3487,7 +3511,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
         <v>90</v>
       </c>
@@ -3495,13 +3519,13 @@
         <v>112</v>
       </c>
       <c r="C15" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>113</v>
       </c>
       <c r="E15" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>114</v>
@@ -3516,7 +3540,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>96</v>
       </c>
@@ -3524,13 +3548,13 @@
         <v>119</v>
       </c>
       <c r="C16" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>120</v>
       </c>
       <c r="E16" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>122</v>
@@ -3545,7 +3569,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
         <v>101</v>
       </c>
@@ -3553,13 +3577,13 @@
         <v>127</v>
       </c>
       <c r="C17" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>113</v>
       </c>
       <c r="E17" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>129</v>
@@ -3574,7 +3598,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
         <v>105</v>
       </c>
@@ -3582,13 +3606,13 @@
         <v>133</v>
       </c>
       <c r="C18" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>134</v>
       </c>
       <c r="E18" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>136</v>
@@ -3603,7 +3627,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
         <v>111</v>
       </c>
@@ -3611,13 +3635,13 @@
         <v>140</v>
       </c>
       <c r="C19" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>141</v>
       </c>
       <c r="E19" s="4">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>143</v>
@@ -3632,7 +3656,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
         <v>115</v>
       </c>
@@ -3640,13 +3664,13 @@
         <v>147</v>
       </c>
       <c r="C20" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>149</v>
       </c>
       <c r="E20" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>150</v>
@@ -3661,7 +3685,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
         <v>121</v>
       </c>
@@ -3669,13 +3693,13 @@
         <v>155</v>
       </c>
       <c r="C21" s="4">
-        <v>46317.0</v>
+        <v>46317</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>156</v>
       </c>
       <c r="E21" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>157</v>
@@ -3690,7 +3714,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
         <v>126</v>
       </c>
@@ -3698,13 +3722,13 @@
         <v>162</v>
       </c>
       <c r="C22" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>163</v>
       </c>
       <c r="E22" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>165</v>
@@ -3719,7 +3743,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
         <v>128</v>
       </c>
@@ -3727,13 +3751,13 @@
         <v>169</v>
       </c>
       <c r="C23" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>171</v>
       </c>
       <c r="E23" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>172</v>
@@ -3748,7 +3772,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
         <v>131</v>
       </c>
@@ -3756,13 +3780,13 @@
         <v>177</v>
       </c>
       <c r="C24" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>178</v>
       </c>
       <c r="E24" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>179</v>
@@ -3777,7 +3801,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
         <v>142</v>
       </c>
@@ -3785,7 +3809,7 @@
         <v>184</v>
       </c>
       <c r="C25" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>185</v>
@@ -3804,7 +3828,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
         <v>148</v>
       </c>
@@ -3812,13 +3836,13 @@
         <v>190</v>
       </c>
       <c r="C26" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>191</v>
       </c>
       <c r="E26" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>193</v>
@@ -3833,7 +3857,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="2" t="s">
         <v>154</v>
       </c>
@@ -3841,13 +3865,13 @@
         <v>196</v>
       </c>
       <c r="C27" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>198</v>
       </c>
       <c r="E27" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>199</v>
@@ -3862,7 +3886,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
         <v>159</v>
       </c>
@@ -3870,13 +3894,13 @@
         <v>202</v>
       </c>
       <c r="C28" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>203</v>
       </c>
       <c r="E28" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>204</v>
@@ -3891,7 +3915,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
         <v>170</v>
       </c>
@@ -3899,13 +3923,13 @@
         <v>209</v>
       </c>
       <c r="C29" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>210</v>
       </c>
       <c r="E29" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>212</v>
@@ -3920,7 +3944,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2" t="s">
         <v>176</v>
       </c>
@@ -3928,13 +3952,13 @@
         <v>217</v>
       </c>
       <c r="C30" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E30" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>219</v>
@@ -3949,7 +3973,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
         <v>181</v>
       </c>
@@ -3957,13 +3981,13 @@
         <v>224</v>
       </c>
       <c r="C31" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>225</v>
       </c>
       <c r="E31" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>226</v>
@@ -3978,7 +4002,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
         <v>187</v>
       </c>
@@ -3986,13 +4010,13 @@
         <v>231</v>
       </c>
       <c r="C32" s="4">
-        <v>46310.0</v>
+        <v>46310</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>233</v>
       </c>
       <c r="E32" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>234</v>
@@ -4007,7 +4031,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
         <v>192</v>
       </c>
@@ -4015,13 +4039,13 @@
         <v>22</v>
       </c>
       <c r="C33" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>191</v>
       </c>
       <c r="E33" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>240</v>
@@ -4036,7 +4060,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
         <v>197</v>
       </c>
@@ -4044,13 +4068,13 @@
         <v>244</v>
       </c>
       <c r="C34" s="4">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>246</v>
       </c>
       <c r="E34" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>247</v>
@@ -4065,7 +4089,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="2" t="s">
         <v>201</v>
       </c>
@@ -4073,13 +4097,13 @@
         <v>252</v>
       </c>
       <c r="C35" s="4">
-        <v>46323.0</v>
+        <v>46323</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>253</v>
       </c>
       <c r="E35" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>255</v>
@@ -4094,7 +4118,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="2" t="s">
         <v>206</v>
       </c>
@@ -4102,13 +4126,13 @@
         <v>259</v>
       </c>
       <c r="C36" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E36" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>261</v>
@@ -4123,7 +4147,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
         <v>211</v>
       </c>
@@ -4131,13 +4155,13 @@
         <v>266</v>
       </c>
       <c r="C37" s="4">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>267</v>
       </c>
       <c r="E37" s="4">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>268</v>
@@ -4152,7 +4176,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
         <v>216</v>
       </c>
@@ -4160,13 +4184,13 @@
         <v>274</v>
       </c>
       <c r="C38" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>191</v>
       </c>
       <c r="E38" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>276</v>
@@ -4181,7 +4205,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
         <v>218</v>
       </c>
@@ -4189,13 +4213,13 @@
         <v>278</v>
       </c>
       <c r="C39" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>191</v>
       </c>
       <c r="E39" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>279</v>
@@ -4210,7 +4234,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
         <v>222</v>
       </c>
@@ -4218,13 +4242,13 @@
         <v>283</v>
       </c>
       <c r="C40" s="4">
-        <v>46283.0</v>
+        <v>46283</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>284</v>
       </c>
       <c r="E40" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>285</v>
@@ -4239,7 +4263,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2" t="s">
         <v>227</v>
       </c>
@@ -4247,13 +4271,13 @@
         <v>289</v>
       </c>
       <c r="C41" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>290</v>
       </c>
       <c r="E41" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>291</v>
@@ -4268,7 +4292,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="2" t="s">
         <v>232</v>
       </c>
@@ -4276,13 +4300,13 @@
         <v>295</v>
       </c>
       <c r="C42" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>296</v>
       </c>
       <c r="E42" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>297</v>
@@ -4297,7 +4321,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="2" t="s">
         <v>237</v>
       </c>
@@ -4305,13 +4329,13 @@
         <v>301</v>
       </c>
       <c r="C43" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>302</v>
       </c>
       <c r="E43" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>303</v>
@@ -4326,7 +4350,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="2" t="s">
         <v>239</v>
       </c>
@@ -4334,13 +4358,13 @@
         <v>307</v>
       </c>
       <c r="C44" s="4">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>308</v>
       </c>
       <c r="E44" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>310</v>
@@ -4355,7 +4379,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="2" t="s">
         <v>245</v>
       </c>
@@ -4363,13 +4387,13 @@
         <v>315</v>
       </c>
       <c r="C45" s="4">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>316</v>
       </c>
       <c r="E45" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>317</v>
@@ -4384,7 +4408,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="2" t="s">
         <v>250</v>
       </c>
@@ -4392,13 +4416,13 @@
         <v>321</v>
       </c>
       <c r="C46" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>322</v>
       </c>
       <c r="E46" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>323</v>
@@ -4413,7 +4437,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="2" t="s">
         <v>254</v>
       </c>
@@ -4421,13 +4445,13 @@
         <v>326</v>
       </c>
       <c r="C47" s="4">
-        <v>46316.0</v>
+        <v>46316</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>327</v>
       </c>
       <c r="E47" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>328</v>
@@ -4442,7 +4466,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="2" t="s">
         <v>260</v>
       </c>
@@ -4450,13 +4474,13 @@
         <v>332</v>
       </c>
       <c r="C48" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>333</v>
       </c>
       <c r="E48" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>334</v>
@@ -4471,7 +4495,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="2" t="s">
         <v>265</v>
       </c>
@@ -4479,13 +4503,13 @@
         <v>340</v>
       </c>
       <c r="C49" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>191</v>
       </c>
       <c r="E49" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>341</v>
@@ -4500,30 +4524,31 @@
         <v>344</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="8" t="s">
         <v>312</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B51"/>
+    <hyperlink ref="B51" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B62"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -4531,495 +4556,495 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="4">
-        <v>46269.0</v>
+        <v>46269</v>
       </c>
       <c r="B2" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4">
-        <v>46270.0</v>
+        <v>46270</v>
       </c>
       <c r="B3" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="4">
-        <v>46271.0</v>
+        <v>46271</v>
       </c>
       <c r="B4" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4">
-        <v>46272.0</v>
+        <v>46272</v>
       </c>
       <c r="B5" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="4">
-        <v>46273.0</v>
+        <v>46273</v>
       </c>
       <c r="B6" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4">
-        <v>46274.0</v>
+        <v>46274</v>
       </c>
       <c r="B7" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="4">
-        <v>46275.0</v>
+        <v>46275</v>
       </c>
       <c r="B8" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="4">
-        <v>46276.0</v>
+        <v>46276</v>
       </c>
       <c r="B9" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="4">
-        <v>46277.0</v>
+        <v>46277</v>
       </c>
       <c r="B10" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="4">
-        <v>46278.0</v>
+        <v>46278</v>
       </c>
       <c r="B11" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="4">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="B12" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="4">
-        <v>46280.0</v>
+        <v>46280</v>
       </c>
       <c r="B13" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="4">
-        <v>46281.0</v>
+        <v>46281</v>
       </c>
       <c r="B14" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="4">
-        <v>46282.0</v>
+        <v>46282</v>
       </c>
       <c r="B15" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="4">
-        <v>46283.0</v>
+        <v>46283</v>
       </c>
       <c r="B16" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="4">
-        <v>46284.0</v>
+        <v>46284</v>
       </c>
       <c r="B17" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="4">
-        <v>46285.0</v>
+        <v>46285</v>
       </c>
       <c r="B18" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="B19" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="4">
-        <v>46287.0</v>
+        <v>46287</v>
       </c>
       <c r="B20" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="4">
-        <v>46288.0</v>
+        <v>46288</v>
       </c>
       <c r="B21" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="4">
-        <v>46289.0</v>
+        <v>46289</v>
       </c>
       <c r="B22" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4">
-        <v>46290.0</v>
+        <v>46290</v>
       </c>
       <c r="B23" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="4">
-        <v>46291.0</v>
+        <v>46291</v>
       </c>
       <c r="B24" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4">
-        <v>46292.0</v>
+        <v>46292</v>
       </c>
       <c r="B25" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="4">
-        <v>46293.0</v>
+        <v>46293</v>
       </c>
       <c r="B26" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="B27" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4">
-        <v>46295.0</v>
+        <v>46295</v>
       </c>
       <c r="B28" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4">
-        <v>46296.0</v>
+        <v>46296</v>
       </c>
       <c r="B29" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4">
-        <v>46297.0</v>
+        <v>46297</v>
       </c>
       <c r="B30" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4">
-        <v>46298.0</v>
+        <v>46298</v>
       </c>
       <c r="B31" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="4">
-        <v>46299.0</v>
+        <v>46299</v>
       </c>
       <c r="B32" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="4">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="B33" s="6">
-        <v>11.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="4">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="B34" s="6">
-        <v>14.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="4">
-        <v>46302.0</v>
+        <v>46302</v>
       </c>
       <c r="B35" s="6">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="4">
-        <v>46303.0</v>
+        <v>46303</v>
       </c>
       <c r="B36" s="6">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="4">
-        <v>46304.0</v>
+        <v>46304</v>
       </c>
       <c r="B37" s="6">
-        <v>15.0</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="4">
-        <v>46305.0</v>
+        <v>46305</v>
       </c>
       <c r="B38" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="4">
-        <v>46306.0</v>
+        <v>46306</v>
       </c>
       <c r="B39" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="4">
-        <v>46307.0</v>
+        <v>46307</v>
       </c>
       <c r="B40" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="4">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="B41" s="6">
-        <v>17.0</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="4">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="B42" s="6">
-        <v>21.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="4">
-        <v>46310.0</v>
+        <v>46310</v>
       </c>
       <c r="B43" s="6">
-        <v>22.0</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="4">
-        <v>46311.0</v>
+        <v>46311</v>
       </c>
       <c r="B44" s="6">
-        <v>25.0</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="4">
-        <v>46312.0</v>
+        <v>46312</v>
       </c>
       <c r="B45" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="4">
-        <v>46313.0</v>
+        <v>46313</v>
       </c>
       <c r="B46" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="4">
-        <v>46314.0</v>
+        <v>46314</v>
       </c>
       <c r="B47" s="6">
-        <v>35.0</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="4">
-        <v>46315.0</v>
+        <v>46315</v>
       </c>
       <c r="B48" s="6">
-        <v>41.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="4">
-        <v>46316.0</v>
+        <v>46316</v>
       </c>
       <c r="B49" s="6">
-        <v>42.0</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="4">
-        <v>46317.0</v>
+        <v>46317</v>
       </c>
       <c r="B50" s="6">
-        <v>44.0</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="4">
-        <v>46318.0</v>
+        <v>46318</v>
       </c>
       <c r="B51" s="6">
-        <v>44.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="4">
-        <v>46319.0</v>
+        <v>46319</v>
       </c>
       <c r="B52" s="6">
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="4">
-        <v>46320.0</v>
+        <v>46320</v>
       </c>
       <c r="B53" s="6">
-        <v>9.0</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="4">
-        <v>46321.0</v>
+        <v>46321</v>
       </c>
       <c r="B54" s="6">
-        <v>48.0</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="4">
-        <v>46322.0</v>
+        <v>46322</v>
       </c>
       <c r="B55" s="6">
-        <v>48.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="4">
-        <v>46323.0</v>
+        <v>46323</v>
       </c>
       <c r="B56" s="6">
-        <v>47.0</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="4">
-        <v>46324.0</v>
+        <v>46324</v>
       </c>
       <c r="B57" s="6">
-        <v>48.0</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="4">
-        <v>46325.0</v>
+        <v>46325</v>
       </c>
       <c r="B58" s="6">
-        <v>44.0</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="4">
-        <v>46326.0</v>
+        <v>46326</v>
       </c>
       <c r="B59" s="6">
-        <v>21.0</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A60" s="4">
-        <v>46327.0</v>
+        <v>46327</v>
       </c>
       <c r="B60" s="6">
-        <v>12.0</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A61" s="4">
-        <v>46328.0</v>
+        <v>46328</v>
       </c>
       <c r="B61" s="6">
-        <v>21.0</v>
-      </c>
-    </row>
-    <row r="62">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A62" s="4">
-        <v>46329.0</v>
+        <v>46329</v>
       </c>
       <c r="B62" s="6">
-        <v>6.0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>